<commit_message>
Importation des fichiers M2
</commit_message>
<xml_diff>
--- a/#000 Coupe NI/Gestion_de_projet RACI Weekly.xlsx
+++ b/#000 Coupe NI/Gestion_de_projet RACI Weekly.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Projet Technique\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\ROBOT NI CONTEST\robotni\#000 Coupe NI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{769EC36B-C92E-425B-A746-0AAA70823E94}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B09CBDC-97D7-4739-B450-D15A050D4F19}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10692" yWindow="2940" windowWidth="17280" windowHeight="8916" tabRatio="705" activeTab="2" xr2:uid="{DA5DF307-7034-4F4E-90E0-F0D7D509C38B}"/>
+    <workbookView xWindow="0" yWindow="2940" windowWidth="17280" windowHeight="8916" tabRatio="705" activeTab="2" xr2:uid="{DA5DF307-7034-4F4E-90E0-F0D7D509C38B}"/>
   </bookViews>
   <sheets>
     <sheet name="RACI" sheetId="2" r:id="rId1"/>
@@ -392,9 +392,6 @@
     <t>#100 - Robot NI</t>
   </si>
   <si>
-    <t>#180 - Armature</t>
-  </si>
-  <si>
     <t>#114 - Sénario JPO: 3 Lidar</t>
   </si>
   <si>
@@ -441,6 +438,9 @@
   </si>
   <si>
     <t>Ce module est independant des autres</t>
+  </si>
+  <si>
+    <t>#180 - Structure Robot</t>
   </si>
 </sst>
 </file>
@@ -1547,10 +1547,10 @@
         <v>29</v>
       </c>
       <c r="T2" s="53" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:21" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1610,10 +1610,10 @@
         <v>29</v>
       </c>
       <c r="T3" s="53" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1675,7 +1675,7 @@
         <v>29</v>
       </c>
       <c r="T4" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:21" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1712,7 +1712,7 @@
         <v>59</v>
       </c>
       <c r="T5" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
@@ -1806,7 +1806,7 @@
         <v>0.87000000000000011</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -2028,7 +2028,7 @@
     <row r="25" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B25" s="16"/>
       <c r="C25" s="34" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D25" s="16"/>
       <c r="E25" s="41"/>
@@ -2341,7 +2341,7 @@
     </row>
     <row r="49" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B49" s="35" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="C49" s="18"/>
       <c r="D49" s="18"/>
@@ -2391,7 +2391,7 @@
         <v>106</v>
       </c>
       <c r="D53" s="23" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E53" s="50" t="s">
         <v>56</v>
@@ -2409,7 +2409,7 @@
         <v>107</v>
       </c>
       <c r="D54" s="23" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E54" s="45" t="s">
         <v>56</v>
@@ -2425,7 +2425,7 @@
         <v>108</v>
       </c>
       <c r="D55" s="23" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E55" s="45" t="s">
         <v>56</v>
@@ -2434,7 +2434,7 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="G55" s="23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.3">
@@ -2484,16 +2484,16 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="G58" s="23" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B59" s="17"/>
       <c r="C59" s="23" t="s">
+        <v>131</v>
+      </c>
+      <c r="D59" s="23" t="s">
         <v>132</v>
-      </c>
-      <c r="D59" s="23" t="s">
-        <v>133</v>
       </c>
       <c r="E59" s="45" t="s">
         <v>56</v>
@@ -2502,7 +2502,7 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="G59" s="23" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="60" spans="2:7" x14ac:dyDescent="0.3">
@@ -2610,7 +2610,7 @@
     <row r="68" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B68" s="17"/>
       <c r="C68" s="23" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D68" s="23" t="s">
         <v>1</v>
@@ -2626,7 +2626,7 @@
     <row r="69" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B69" s="17"/>
       <c r="C69" s="23" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D69" s="23" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Upload Datasheet Raspberry PI
</commit_message>
<xml_diff>
--- a/#000 Coupe NI/Gestion_de_projet RACI Weekly.xlsx
+++ b/#000 Coupe NI/Gestion_de_projet RACI Weekly.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\ROBOT NI CONTEST\robotni\#000 Coupe NI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B09CBDC-97D7-4739-B450-D15A050D4F19}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD30065A-75E4-4CF5-8B7F-7EE781DC9B2B}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2940" windowWidth="17280" windowHeight="8916" tabRatio="705" activeTab="2" xr2:uid="{DA5DF307-7034-4F4E-90E0-F0D7D509C38B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="705" activeTab="2" xr2:uid="{DA5DF307-7034-4F4E-90E0-F0D7D509C38B}"/>
   </bookViews>
   <sheets>
     <sheet name="RACI" sheetId="2" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="136">
   <si>
     <t xml:space="preserve">Semaine </t>
   </si>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C4" s="46">
         <f ca="1">(SUM(E12,C5,E18))/3</f>
-        <v>0.23571428571428574</v>
+        <v>0.3428571428571428</v>
       </c>
       <c r="D4" s="20"/>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C5" s="42">
         <f>(SUM(E29,E32,E35,E39,E43,E21,E46))/7</f>
-        <v>0.45714285714285718</v>
+        <v>0.52857142857142858</v>
       </c>
       <c r="D5" s="18"/>
     </row>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="C6" s="44">
         <f>(SUM(E67,E61,E52))/3</f>
-        <v>0.87000000000000011</v>
+        <v>1</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>134</v>
@@ -1865,7 +1865,7 @@
       <c r="D12" s="20"/>
       <c r="E12" s="40">
         <f ca="1">SUMIF(E13:F16,"Done",F13:F16)</f>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="F12" s="28"/>
       <c r="G12" s="20"/>
@@ -1878,7 +1878,9 @@
       <c r="D13" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="E13" s="48"/>
+      <c r="E13" s="48" t="s">
+        <v>60</v>
+      </c>
       <c r="F13" s="30">
         <v>0.25</v>
       </c>
@@ -1893,7 +1895,7 @@
         <v>2</v>
       </c>
       <c r="E14" s="48" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F14" s="30">
         <v>0.25</v>
@@ -2265,7 +2267,7 @@
       <c r="D43" s="18"/>
       <c r="E43" s="43">
         <f>SUMIF(E44:E45,"Done",F44:F45)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F43" s="22"/>
       <c r="G43" s="18"/>
@@ -2276,7 +2278,9 @@
         <v>97</v>
       </c>
       <c r="D44" s="16"/>
-      <c r="E44" s="41"/>
+      <c r="E44" s="47" t="s">
+        <v>56</v>
+      </c>
       <c r="F44" s="31">
         <v>0.5</v>
       </c>
@@ -2380,7 +2384,7 @@
       <c r="D52" s="21"/>
       <c r="E52" s="44">
         <f>SUMIF(E53:E59,"Done",F53:F59)</f>
-        <v>0.8600000000000001</v>
+        <v>1</v>
       </c>
       <c r="F52" s="24"/>
       <c r="G52" s="21"/>
@@ -2478,7 +2482,7 @@
         <v>2</v>
       </c>
       <c r="E58" s="45" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F58" s="32">
         <v>0.14000000000000001</v>
@@ -2521,7 +2525,7 @@
       <c r="D61" s="19"/>
       <c r="E61" s="44">
         <f>SUMIF(E62:E65,"Done",F62:F65)</f>
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="F61" s="24"/>
       <c r="G61" s="19"/>
@@ -2531,8 +2535,12 @@
       <c r="C62" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="D62" s="17"/>
-      <c r="E62" s="49"/>
+      <c r="D62" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="E62" s="50" t="s">
+        <v>56</v>
+      </c>
       <c r="F62" s="33">
         <v>0.25</v>
       </c>

</xml_diff>

<commit_message>
PCB V3 + Weekly
</commit_message>
<xml_diff>
--- a/#000 Coupe NI/Gestion_de_projet RACI Weekly.xlsx
+++ b/#000 Coupe NI/Gestion_de_projet RACI Weekly.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\ROBOT NI CONTEST\robotni\#000 Coupe NI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61C4DC8A-8DAA-45CF-9BA2-57D07EC18F99}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CBE2D02-A8FA-4515-85D0-D13A11CEE50C}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2868" windowWidth="17280" windowHeight="8916" tabRatio="705" activeTab="2" xr2:uid="{DA5DF307-7034-4F4E-90E0-F0D7D509C38B}"/>
+    <workbookView xWindow="1608" yWindow="348" windowWidth="17280" windowHeight="8916" tabRatio="705" activeTab="2" xr2:uid="{DA5DF307-7034-4F4E-90E0-F0D7D509C38B}"/>
   </bookViews>
   <sheets>
     <sheet name="RACI" sheetId="2" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="148">
   <si>
     <t xml:space="preserve">Semaine </t>
   </si>
@@ -335,9 +335,6 @@
     <t>Nicolas COURT</t>
   </si>
   <si>
-    <t>Quentin BAUDIN</t>
-  </si>
-  <si>
     <t>#014 - Weekly Report</t>
   </si>
   <si>
@@ -468,6 +465,18 @@
   </si>
   <si>
     <t>IMPORTANT: ABSENCE DE REGLES NI</t>
+  </si>
+  <si>
+    <t>Rebuild</t>
+  </si>
+  <si>
+    <t>Quentin BAUDIN -&gt; Jason PUEL</t>
+  </si>
+  <si>
+    <t>PCB V3</t>
+  </si>
+  <si>
+    <t>Testing  Code LabVIew</t>
   </si>
 </sst>
 </file>
@@ -673,7 +682,7 @@
     <xf numFmtId="0" fontId="3" fillId="16" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -780,13 +789,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="20 % - Accent1" xfId="3" builtinId="30"/>
@@ -1451,7 +1461,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2827ADE7-BE37-4A6E-A5BE-B763B36190AE}">
   <sheetPr codeName="Feuil2"/>
-  <dimension ref="A1:AA8"/>
+  <dimension ref="A1:AD11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="5" width="16.109375" customWidth="1"/>
@@ -1466,7 +1476,7 @@
     <col min="26" max="26" width="7.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1548,8 +1558,17 @@
       <c r="AA1" s="1">
         <v>43577</v>
       </c>
-    </row>
-    <row r="2" spans="1:27" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AB1" s="1">
+        <v>43584</v>
+      </c>
+      <c r="AC1" s="1">
+        <v>43591</v>
+      </c>
+      <c r="AD1" s="1">
+        <v>43598</v>
+      </c>
+    </row>
+    <row r="2" spans="1:30" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1608,29 +1627,38 @@
         <v>29</v>
       </c>
       <c r="T2" s="52" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="U2" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="V2" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="V2" s="2" t="s">
-        <v>133</v>
-      </c>
       <c r="W2" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="Y2" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="Z2" s="58"/>
+        <v>139</v>
+      </c>
+      <c r="Z2" s="56"/>
       <c r="AA2" s="3" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>139</v>
+      </c>
+      <c r="AB2" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="AC2" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="AD2" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1687,29 +1715,38 @@
         <v>29</v>
       </c>
       <c r="T3" s="52" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="W3" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="Y3" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="Z3" s="58"/>
+        <v>139</v>
+      </c>
+      <c r="Z3" s="56"/>
       <c r="AA3" s="3" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="4" spans="1:27" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>139</v>
+      </c>
+      <c r="AB3" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="AC3" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="AD3" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="4" spans="1:30" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1768,27 +1805,31 @@
         <v>29</v>
       </c>
       <c r="T4" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="U4" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="W4" s="2"/>
       <c r="X4" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="Y4" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="Z4" s="58"/>
-      <c r="AA4" s="3" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="5" spans="1:27" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>139</v>
+      </c>
+      <c r="Z4" s="56"/>
+      <c r="AB4" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="AC4" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="AD4" s="59"/>
+    </row>
+    <row r="5" spans="1:30" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -1823,7 +1864,7 @@
       </c>
       <c r="S5" s="55"/>
       <c r="T5" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="U5" s="3" t="s">
         <v>31</v>
@@ -1832,17 +1873,29 @@
         <v>31</v>
       </c>
       <c r="W5" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="X5" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="X5" s="3" t="s">
-        <v>141</v>
-      </c>
       <c r="Y5" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="Z5" s="58"/>
-    </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+      <c r="Z5" s="56"/>
+      <c r="AA5" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="AB5" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="AC5" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="AD5" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
       <c r="F6" t="s">
         <v>22</v>
       </c>
@@ -1853,15 +1906,18 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
       <c r="F7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
       <c r="F8" t="s">
         <v>24</v>
       </c>
+    </row>
+    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="AB11" s="59"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1885,12 +1941,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
     </row>
     <row r="3" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B3" s="27" t="s">
@@ -1910,19 +1966,19 @@
       </c>
       <c r="C4" s="45">
         <f ca="1">(SUM(E10,C5,E15))/3</f>
-        <v>0.54952380952380953</v>
+        <v>0.53523809523809529</v>
       </c>
       <c r="D4" s="36" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B5" s="35" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C5" s="41">
         <f>(SUM(E26,E29,E32,E36,E40,E18,E43))/7</f>
-        <v>0.64857142857142858</v>
+        <v>0.60571428571428576</v>
       </c>
       <c r="D5" s="18"/>
     </row>
@@ -1935,16 +1991,16 @@
         <v>0.95333333333333325</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="56" t="s">
+      <c r="B8" s="57" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="56"/>
-      <c r="D8" s="56"/>
-      <c r="E8" s="56"/>
+      <c r="C8" s="57"/>
+      <c r="D8" s="57"/>
+      <c r="E8" s="57"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
@@ -1985,7 +2041,7 @@
         <v>78</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E11" s="47" t="s">
         <v>56</v>
@@ -2001,7 +2057,7 @@
         <v>79</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E12" s="47" t="s">
         <v>56</v>
@@ -2014,7 +2070,7 @@
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B13" s="15"/>
       <c r="C13" s="29" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D13" s="29" t="s">
         <v>1</v>
@@ -2052,7 +2108,7 @@
       <c r="B16" s="15"/>
       <c r="C16" s="15"/>
       <c r="D16" s="29" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E16" s="54" t="s">
         <v>59</v>
@@ -2078,7 +2134,7 @@
       <c r="D18" s="18"/>
       <c r="E18" s="41">
         <f>SUMIF(E19:E24,"Done",F19:F24)</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="F18" s="22"/>
       <c r="G18" s="18"/>
@@ -2126,10 +2182,12 @@
     <row r="22" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B22" s="16"/>
       <c r="C22" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D22" s="16"/>
-      <c r="E22" s="40"/>
+      <c r="E22" s="40" t="s">
+        <v>56</v>
+      </c>
       <c r="F22" s="50">
         <v>0.2</v>
       </c>
@@ -2152,7 +2210,7 @@
     <row r="24" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B24" s="16"/>
       <c r="C24" s="34" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D24" s="34"/>
       <c r="E24" s="40"/>
@@ -2367,7 +2425,7 @@
       <c r="D40" s="18"/>
       <c r="E40" s="42">
         <f>SUMIF(E41:E42,"Done",F41:F42)</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F40" s="22"/>
       <c r="G40" s="18"/>
@@ -2392,15 +2450,17 @@
         <v>95</v>
       </c>
       <c r="D42" s="34" t="s">
-        <v>100</v>
+        <v>145</v>
       </c>
       <c r="E42" s="40" t="s">
-        <v>56</v>
+        <v>144</v>
       </c>
       <c r="F42" s="31">
         <v>0.5</v>
       </c>
-      <c r="G42" s="16"/>
+      <c r="G42" s="16" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B43" s="35" t="s">
@@ -2447,7 +2507,7 @@
     </row>
     <row r="46" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B46" s="35" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C46" s="18"/>
       <c r="D46" s="18"/>
@@ -2461,7 +2521,7 @@
     <row r="47" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B47" s="16"/>
       <c r="C47" s="34" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D47" s="16"/>
       <c r="E47" s="46" t="s">
@@ -2496,10 +2556,10 @@
     <row r="50" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B50" s="17"/>
       <c r="C50" s="23" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E50" s="49" t="s">
         <v>56</v>
@@ -2508,16 +2568,16 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="G50" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="51" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B51" s="17"/>
       <c r="C51" s="23" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E51" s="44" t="s">
         <v>56</v>
@@ -2530,10 +2590,10 @@
     <row r="52" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B52" s="17"/>
       <c r="C52" s="23" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D52" s="23" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E52" s="44" t="s">
         <v>56</v>
@@ -2542,13 +2602,13 @@
         <v>0.12</v>
       </c>
       <c r="G52" s="23" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="53" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B53" s="17"/>
       <c r="C53" s="23" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D53" s="23" t="s">
         <v>2</v>
@@ -2564,7 +2624,7 @@
     <row r="54" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B54" s="17"/>
       <c r="C54" s="23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D54" s="23" t="s">
         <v>2</v>
@@ -2580,7 +2640,7 @@
     <row r="55" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B55" s="17"/>
       <c r="C55" s="23" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D55" s="23" t="s">
         <v>2</v>
@@ -2592,16 +2652,16 @@
         <v>0.12</v>
       </c>
       <c r="G55" s="23" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B56" s="17"/>
       <c r="C56" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="D56" s="23" t="s">
         <v>124</v>
-      </c>
-      <c r="D56" s="23" t="s">
-        <v>125</v>
       </c>
       <c r="E56" s="44" t="s">
         <v>56</v>
@@ -2610,17 +2670,17 @@
         <v>0.12</v>
       </c>
       <c r="G56" s="23" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B57" s="17"/>
       <c r="C57" s="23" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D57" s="23"/>
       <c r="E57" s="44" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F57" s="32">
         <v>0.12</v>
@@ -2637,7 +2697,7 @@
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B59" s="21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C59" s="19"/>
       <c r="D59" s="19"/>
@@ -2651,7 +2711,7 @@
     <row r="60" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B60" s="17"/>
       <c r="C60" s="23" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D60" s="23" t="s">
         <v>1</v>
@@ -2667,7 +2727,7 @@
     <row r="61" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B61" s="17"/>
       <c r="C61" s="23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D61" s="23" t="s">
         <v>40</v>
@@ -2683,7 +2743,7 @@
     <row r="62" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B62" s="17"/>
       <c r="C62" s="23" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D62" s="23" t="s">
         <v>98</v>
@@ -2699,7 +2759,7 @@
     <row r="63" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B63" s="17"/>
       <c r="C63" s="23" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D63" s="23" t="s">
         <v>1</v>
@@ -2722,7 +2782,7 @@
     </row>
     <row r="65" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B65" s="21" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C65" s="19"/>
       <c r="D65" s="19"/>
@@ -2736,7 +2796,7 @@
     <row r="66" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B66" s="17"/>
       <c r="C66" s="23" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D66" s="23" t="s">
         <v>1</v>
@@ -2752,7 +2812,7 @@
     <row r="67" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B67" s="17"/>
       <c r="C67" s="23" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D67" s="23" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Gestion de projet + Pitch2 Poster
</commit_message>
<xml_diff>
--- a/#000 Coupe NI/Gestion_de_projet RACI Weekly.xlsx
+++ b/#000 Coupe NI/Gestion_de_projet RACI Weekly.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\ROBOT NI CONTEST\robotni\#000 Coupe NI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CBE2D02-A8FA-4515-85D0-D13A11CEE50C}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9234464C-36CA-49A6-9E0D-08446F404540}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1608" yWindow="348" windowWidth="17280" windowHeight="8916" tabRatio="705" activeTab="2" xr2:uid="{DA5DF307-7034-4F4E-90E0-F0D7D509C38B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="705" activeTab="3" xr2:uid="{DA5DF307-7034-4F4E-90E0-F0D7D509C38B}"/>
   </bookViews>
   <sheets>
     <sheet name="RACI" sheetId="2" r:id="rId1"/>
     <sheet name="Weekly" sheetId="1" r:id="rId2"/>
     <sheet name="Gestion des fichiers" sheetId="3" r:id="rId3"/>
+    <sheet name="Code Labview" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="184">
   <si>
     <t xml:space="preserve">Semaine </t>
   </si>
@@ -206,9 +207,6 @@
     <t>Done</t>
   </si>
   <si>
-    <t>Adiren</t>
-  </si>
-  <si>
     <t>Teste/Reparation du raspberry</t>
   </si>
   <si>
@@ -278,15 +276,6 @@
     <t xml:space="preserve">#111 - Code Concour </t>
   </si>
   <si>
-    <t>#112 - Sénario JPO: 1</t>
-  </si>
-  <si>
-    <t>#113 - Sénario JPO: 2</t>
-  </si>
-  <si>
-    <t>#115 - Sénario JPO: 4</t>
-  </si>
-  <si>
     <t>#121 - Datasheet et Composant</t>
   </si>
   <si>
@@ -305,9 +294,6 @@
     <t>#142 - Model 3D</t>
   </si>
   <si>
-    <t>#143 - Découpe Laser</t>
-  </si>
-  <si>
     <t>#151 - Datasheet et Composant</t>
   </si>
   <si>
@@ -320,9 +306,6 @@
     <t>#161 - Datasheet et Composant</t>
   </si>
   <si>
-    <t>#162 - Eagle</t>
-  </si>
-  <si>
     <t>#171 - Datasheet et Composant</t>
   </si>
   <si>
@@ -380,9 +363,6 @@
     <t>#100 - Robot NI</t>
   </si>
   <si>
-    <t>#114 - Sénario JPO: 3 Lidar</t>
-  </si>
-  <si>
     <t>Demander a Willi du sevice info + designier responsable</t>
   </si>
   <si>
@@ -419,9 +399,6 @@
     <t>#180 - Structure Robot</t>
   </si>
   <si>
-    <t>#116 - Sénario JPO: 5</t>
-  </si>
-  <si>
     <t>Etude du code  LabView</t>
   </si>
   <si>
@@ -477,13 +454,145 @@
   </si>
   <si>
     <t>Testing  Code LabVIew</t>
+  </si>
+  <si>
+    <t>#155 - Moteur trap</t>
+  </si>
+  <si>
+    <t>#156 - Moteur manege</t>
+  </si>
+  <si>
+    <t>#154 - Diode Détecteur couleur</t>
+  </si>
+  <si>
+    <t>#112 - Sénario JPO: Lidar</t>
+  </si>
+  <si>
+    <t>Tout le monde</t>
+  </si>
+  <si>
+    <t>#164 - Faire imprimer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analise </t>
+  </si>
+  <si>
+    <t>Attente de la fin de l'analise</t>
+  </si>
+  <si>
+    <t>#162 - Correction et amelioration</t>
+  </si>
+  <si>
+    <t>#163 - Eagle</t>
+  </si>
+  <si>
+    <t>Responsable</t>
+  </si>
+  <si>
+    <t>Main_RT_V2</t>
+  </si>
+  <si>
+    <t>Sous_VI_Avancer</t>
+  </si>
+  <si>
+    <t>non</t>
+  </si>
+  <si>
+    <t>Jason PUEL et Justin Furio</t>
+  </si>
+  <si>
+    <t>Sous_VI_RT_recule</t>
+  </si>
+  <si>
+    <t>Sous_VI_RT_Virage</t>
+  </si>
+  <si>
+    <t>Sous_VI_RT_Sceaux</t>
+  </si>
+  <si>
+    <t>Sous_VI_RT_trieur-balles</t>
+  </si>
+  <si>
+    <t>Florian GUIGAL et Justin Furio</t>
+  </si>
+  <si>
+    <t>Sous_VI_Bras</t>
+  </si>
+  <si>
+    <t>Sous_VI_acp_ligne</t>
+  </si>
+  <si>
+    <t>Sous_VI_correction</t>
+  </si>
+  <si>
+    <t>Sous_VI_moteurs</t>
+  </si>
+  <si>
+    <t>Moteur_trieur_balle_adrien</t>
+  </si>
+  <si>
+    <t>Adrien</t>
+  </si>
+  <si>
+    <t>trieur_trappe</t>
+  </si>
+  <si>
+    <t>trieur_Couleur</t>
+  </si>
+  <si>
+    <t>Sous_VI_RT_Lanceur</t>
+  </si>
+  <si>
+    <t>Sous_VI_distributeur_lanceur</t>
+  </si>
+  <si>
+    <t>Sous_VI_moteur_roue_lanceur</t>
+  </si>
+  <si>
+    <t>enum_Main_RT_V2</t>
+  </si>
+  <si>
+    <t>enum_RT_Virage</t>
+  </si>
+  <si>
+    <t>enum_RT_Sceaux</t>
+  </si>
+  <si>
+    <t>enum_RT_recule</t>
+  </si>
+  <si>
+    <t>enum_RT_bras</t>
+  </si>
+  <si>
+    <t>enum_VI_RT_trieur-balles</t>
+  </si>
+  <si>
+    <t>enum_lanceur</t>
+  </si>
+  <si>
+    <t>enum_distributeur_lanceur</t>
+  </si>
+  <si>
+    <t>enum_moteur_lanceur</t>
+  </si>
+  <si>
+    <t>niveau :</t>
+  </si>
+  <si>
+    <t>nom du VI</t>
+  </si>
+  <si>
+    <t>Enum associé</t>
+  </si>
+  <si>
+    <t>Préparation poster</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -523,6 +632,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -682,7 +797,7 @@
     <xf numFmtId="0" fontId="3" fillId="16" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -790,13 +905,14 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="20 % - Accent1" xfId="3" builtinId="30"/>
@@ -851,8 +967,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{32F8ADCA-7BE8-4A17-965F-3A7BAA9A6A31}" name="Tableau2" displayName="Tableau2" ref="B9:G68" totalsRowShown="0">
-  <autoFilter ref="B9:G68" xr:uid="{5E9D7C67-1BBD-465F-A208-D11E9B7D938B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{32F8ADCA-7BE8-4A17-965F-3A7BAA9A6A31}" name="Tableau2" displayName="Tableau2" ref="B9:G74" totalsRowShown="0">
+  <autoFilter ref="B9:G74" xr:uid="{5E9D7C67-1BBD-465F-A208-D11E9B7D938B}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{331D23FA-9A32-4E23-A796-24563384C5B8}" name="Partie Projet"/>
     <tableColumn id="2" xr3:uid="{73E2A53B-9F6D-48BD-9CD1-4D3FFFEEA257}" name="Sous taches"/>
@@ -1461,7 +1577,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2827ADE7-BE37-4A6E-A5BE-B763B36190AE}">
   <sheetPr codeName="Feuil2"/>
-  <dimension ref="A1:AD11"/>
+  <dimension ref="A1:AF11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="5" width="16.109375" customWidth="1"/>
@@ -1474,9 +1590,10 @@
     <col min="17" max="17" width="13.5546875" customWidth="1"/>
     <col min="19" max="19" width="7.5546875" customWidth="1"/>
     <col min="26" max="26" width="7.21875" customWidth="1"/>
+    <col min="31" max="31" width="9.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1567,8 +1684,14 @@
       <c r="AD1" s="1">
         <v>43598</v>
       </c>
-    </row>
-    <row r="2" spans="1:30" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AE1" s="1">
+        <v>43601</v>
+      </c>
+      <c r="AF1" s="1">
+        <v>43605</v>
+      </c>
+    </row>
+    <row r="2" spans="1:32" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1621,44 +1744,47 @@
         <v>27</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="S2" s="52" t="s">
         <v>29</v>
       </c>
       <c r="T2" s="52" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="U2" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="W2" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="V2" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="W2" s="3" t="s">
-        <v>139</v>
-      </c>
       <c r="X2" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="Y2" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="Z2" s="56"/>
       <c r="AA2" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="AB2" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="AC2" s="2" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="AD2" s="3" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="3" spans="1:30" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>138</v>
+      </c>
+      <c r="AE2" s="56" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="3" spans="1:32" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1709,44 +1835,47 @@
         <v>11</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="S3" s="52" t="s">
         <v>29</v>
       </c>
       <c r="T3" s="52" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="W3" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="Y3" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="Z3" s="56"/>
       <c r="AA3" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="AB3" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="AC3" s="2" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="AD3" s="2" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="4" spans="1:30" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+      <c r="AE3" s="56" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1805,31 +1934,36 @@
         <v>29</v>
       </c>
       <c r="T4" s="4" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="U4" s="3" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="W4" s="2"/>
       <c r="X4" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="Y4" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="Z4" s="56"/>
       <c r="AB4" s="3" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="AC4" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="AD4" s="59"/>
-    </row>
-    <row r="5" spans="1:30" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+      <c r="AD4" s="56" t="s">
+        <v>183</v>
+      </c>
+      <c r="AE4" s="56" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -1860,11 +1994,11 @@
         <v>27</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="S5" s="55"/>
       <c r="T5" s="4" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="U5" s="3" t="s">
         <v>31</v>
@@ -1873,29 +2007,32 @@
         <v>31</v>
       </c>
       <c r="W5" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="X5" s="3" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="Y5" s="3" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="Z5" s="56"/>
       <c r="AA5" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="AB5" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="AC5" s="2" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="AD5" s="2" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+      <c r="AE5" s="56" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
       <c r="F6" t="s">
         <v>22</v>
       </c>
@@ -1906,18 +2043,18 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.3">
       <c r="F7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
       <c r="F8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="AB11" s="59"/>
+    <row r="11" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="AB11" s="57"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1928,7 +2065,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6C9BC92-4796-4401-A0F6-67380B3C0ACF}">
   <sheetPr codeName="Feuil3"/>
-  <dimension ref="B2:G73"/>
+  <dimension ref="B2:G79"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.88671875" customWidth="1"/>
@@ -1941,73 +2078,73 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B2" s="58" t="s">
-        <v>60</v>
-      </c>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
+      <c r="B2" s="59" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
     </row>
     <row r="3" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B3" s="27" t="s">
         <v>52</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D3" s="27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E3" s="25"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B4" s="36" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C4" s="45">
         <f ca="1">(SUM(E10,C5,E15))/3</f>
-        <v>0.53523809523809529</v>
+        <v>0.56285714285714283</v>
       </c>
       <c r="D4" s="36" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B5" s="35" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="C5" s="41">
-        <f>(SUM(E26,E29,E32,E36,E40,E18,E43))/7</f>
-        <v>0.60571428571428576</v>
+        <f>(SUM(E22,E26,E30,E34,E42,E18,E48))/7</f>
+        <v>0.68857142857142861</v>
       </c>
       <c r="D5" s="18"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B6" s="21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C6" s="43">
-        <f>(SUM(E65,E59,E49))/3</f>
+        <f>(SUM(E71,E65,E55))/3</f>
         <v>0.95333333333333325</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="57" t="s">
+      <c r="B8" s="58" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="57"/>
-      <c r="D8" s="57"/>
-      <c r="E8" s="57"/>
+      <c r="C8" s="58"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="58"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>52</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
         <v>55</v>
@@ -2016,15 +2153,15 @@
         <v>53</v>
       </c>
       <c r="F9" s="26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B10" s="36" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C10" s="20"/>
       <c r="D10" s="20"/>
@@ -2038,10 +2175,10 @@
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B11" s="15"/>
       <c r="C11" s="29" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="E11" s="47" t="s">
         <v>56</v>
@@ -2054,10 +2191,10 @@
     <row r="12" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B12" s="15"/>
       <c r="C12" s="29" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="E12" s="47" t="s">
         <v>56</v>
@@ -2070,7 +2207,7 @@
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B13" s="15"/>
       <c r="C13" s="29" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D13" s="29" t="s">
         <v>1</v>
@@ -2093,7 +2230,7 @@
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B15" s="36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C15" s="20"/>
       <c r="D15" s="20"/>
@@ -2108,10 +2245,10 @@
       <c r="B16" s="15"/>
       <c r="C16" s="15"/>
       <c r="D16" s="29" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="E16" s="54" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F16" s="37">
         <v>1</v>
@@ -2128,13 +2265,13 @@
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B18" s="35" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C18" s="18"/>
       <c r="D18" s="18"/>
       <c r="E18" s="41">
-        <f>SUMIF(E19:E24,"Done",F19:F24)</f>
-        <v>0.4</v>
+        <f>SUMIF(E19:E20,"Done",F19:F20)</f>
+        <v>1</v>
       </c>
       <c r="F18" s="22"/>
       <c r="G18" s="18"/>
@@ -2142,80 +2279,79 @@
     <row r="19" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B19" s="16"/>
       <c r="C19" s="34" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="E19" s="40"/>
+        <v>144</v>
+      </c>
+      <c r="E19" s="40" t="s">
+        <v>56</v>
+      </c>
       <c r="F19" s="50">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="G19" s="16"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B20" s="16"/>
       <c r="C20" s="34" t="s">
-        <v>81</v>
-      </c>
-      <c r="D20" s="16"/>
+        <v>143</v>
+      </c>
+      <c r="D20" s="34" t="s">
+        <v>63</v>
+      </c>
       <c r="E20" s="46" t="s">
         <v>56</v>
       </c>
       <c r="F20" s="50">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="G20" s="16"/>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B21" s="16"/>
-      <c r="C21" s="34" t="s">
-        <v>82</v>
-      </c>
+      <c r="C21" s="34"/>
       <c r="D21" s="16"/>
       <c r="E21" s="40"/>
-      <c r="F21" s="50">
-        <v>0.2</v>
-      </c>
+      <c r="F21" s="31"/>
       <c r="G21" s="16"/>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B22" s="16"/>
-      <c r="C22" s="34" t="s">
-        <v>115</v>
-      </c>
-      <c r="D22" s="16"/>
-      <c r="E22" s="40" t="s">
-        <v>56</v>
-      </c>
-      <c r="F22" s="50">
-        <v>0.2</v>
-      </c>
-      <c r="G22" s="16"/>
+      <c r="B22" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="41">
+        <f>SUMIF(E23:E24,"Done",F23:F24)</f>
+        <v>0.5</v>
+      </c>
+      <c r="F22" s="22"/>
+      <c r="G22" s="18"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B23" s="16"/>
       <c r="C23" s="34" t="s">
-        <v>83</v>
-      </c>
-      <c r="D23" s="34" t="s">
-        <v>64</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="D23" s="16"/>
       <c r="E23" s="40"/>
-      <c r="F23" s="50">
-        <v>0.2</v>
+      <c r="F23" s="31">
+        <v>0.5</v>
       </c>
       <c r="G23" s="16"/>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B24" s="16"/>
       <c r="C24" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="D24" s="34"/>
-      <c r="E24" s="40"/>
-      <c r="F24" s="50">
-        <v>0.2</v>
+        <v>81</v>
+      </c>
+      <c r="D24" s="16"/>
+      <c r="E24" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F24" s="31">
+        <v>0.5</v>
       </c>
       <c r="G24" s="16"/>
     </row>
@@ -2235,7 +2371,7 @@
       <c r="D26" s="18"/>
       <c r="E26" s="41">
         <f>SUMIF(E27:E28,"Done",F27:F28)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F26" s="22"/>
       <c r="G26" s="18"/>
@@ -2243,10 +2379,12 @@
     <row r="27" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B27" s="16"/>
       <c r="C27" s="34" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D27" s="16"/>
-      <c r="E27" s="40"/>
+      <c r="E27" s="40" t="s">
+        <v>56</v>
+      </c>
       <c r="F27" s="31">
         <v>0.5</v>
       </c>
@@ -2255,9 +2393,11 @@
     <row r="28" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B28" s="16"/>
       <c r="C28" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="D28" s="16"/>
+        <v>83</v>
+      </c>
+      <c r="D28" s="34" t="s">
+        <v>1</v>
+      </c>
       <c r="E28" s="40" t="s">
         <v>56</v>
       </c>
@@ -2267,527 +2407,509 @@
       <c r="G28" s="16"/>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B29" s="35" t="s">
+      <c r="B29" s="16"/>
+      <c r="C29" s="34"/>
+      <c r="D29" s="34"/>
+      <c r="E29" s="40"/>
+      <c r="F29" s="31"/>
+      <c r="G29" s="16"/>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B30" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="41">
-        <f>SUMIF(E30:E31,"Done",F30:F31)</f>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="41">
+        <f>SUMIF(E31:E32,"Done",F31:F32)</f>
         <v>0.5</v>
       </c>
-      <c r="F29" s="22"/>
-      <c r="G29" s="18"/>
-    </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B30" s="16"/>
-      <c r="C30" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="D30" s="16"/>
-      <c r="E30" s="40"/>
-      <c r="F30" s="31">
-        <v>0.5</v>
-      </c>
-      <c r="G30" s="16"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="18"/>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B31" s="16"/>
       <c r="C31" s="34" t="s">
-        <v>87</v>
-      </c>
-      <c r="D31" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="E31" s="40" t="s">
-        <v>56</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="D31" s="16"/>
+      <c r="E31" s="40"/>
       <c r="F31" s="31">
         <v>0.5</v>
       </c>
       <c r="G31" s="16"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B32" s="35" t="s">
-        <v>73</v>
-      </c>
-      <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="41">
-        <f>SUMIF(E33:E35,"Done",F33:F35)</f>
-        <v>0.67</v>
-      </c>
-      <c r="F32" s="22"/>
-      <c r="G32" s="18"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="D32" s="16"/>
+      <c r="E32" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F32" s="31">
+        <v>0.5</v>
+      </c>
+      <c r="G32" s="16"/>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B33" s="16"/>
-      <c r="C33" s="34" t="s">
-        <v>88</v>
-      </c>
+      <c r="C33" s="34"/>
       <c r="D33" s="16"/>
-      <c r="E33" s="40"/>
-      <c r="F33" s="31">
-        <v>0.33</v>
-      </c>
+      <c r="E33" s="46"/>
+      <c r="F33" s="31"/>
       <c r="G33" s="16"/>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B34" s="16"/>
-      <c r="C34" s="34" t="s">
-        <v>89</v>
-      </c>
-      <c r="D34" s="16"/>
-      <c r="E34" s="40" t="s">
-        <v>56</v>
-      </c>
-      <c r="F34" s="31">
-        <v>0.33</v>
-      </c>
-      <c r="G34" s="16"/>
+      <c r="B34" s="35" t="s">
+        <v>73</v>
+      </c>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="42">
+        <f>SUMIF(E35:E40,"Done",F35:F40)</f>
+        <v>0.82000000000000006</v>
+      </c>
+      <c r="F34" s="22"/>
+      <c r="G34" s="18"/>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B35" s="16"/>
       <c r="C35" s="34" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D35" s="16"/>
-      <c r="E35" s="46" t="s">
+      <c r="E35" s="40"/>
+      <c r="F35" s="31">
+        <v>0.18</v>
+      </c>
+      <c r="G35" s="16"/>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B36" s="16"/>
+      <c r="C36" s="34" t="s">
+        <v>87</v>
+      </c>
+      <c r="D36" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="E36" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="F35" s="31">
-        <v>0.34</v>
-      </c>
-      <c r="G35" s="16"/>
-    </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B36" s="35" t="s">
-        <v>74</v>
-      </c>
-      <c r="C36" s="18"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="42">
-        <f>SUMIF(E37:E39,"Done",F37:F39)</f>
-        <v>0.67</v>
-      </c>
-      <c r="F36" s="22"/>
-      <c r="G36" s="18"/>
+      <c r="F36" s="31">
+        <v>0.16</v>
+      </c>
+      <c r="G36" s="16"/>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B37" s="16"/>
       <c r="C37" s="34" t="s">
-        <v>91</v>
-      </c>
-      <c r="D37" s="16"/>
-      <c r="E37" s="40"/>
+        <v>88</v>
+      </c>
+      <c r="D37" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="E37" s="46" t="s">
+        <v>56</v>
+      </c>
       <c r="F37" s="31">
-        <v>0.33</v>
+        <v>0.16500000000000001</v>
       </c>
       <c r="G37" s="16"/>
     </row>
     <row r="38" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B38" s="16"/>
       <c r="C38" s="34" t="s">
-        <v>92</v>
+        <v>142</v>
       </c>
       <c r="D38" s="34" t="s">
-        <v>98</v>
-      </c>
-      <c r="E38" s="40" t="s">
+        <v>40</v>
+      </c>
+      <c r="E38" s="46" t="s">
         <v>56</v>
       </c>
       <c r="F38" s="31">
-        <v>0.33</v>
+        <v>0.16500000000000001</v>
       </c>
       <c r="G38" s="16"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B39" s="16"/>
       <c r="C39" s="34" t="s">
-        <v>93</v>
+        <v>140</v>
       </c>
       <c r="D39" s="34" t="s">
-        <v>98</v>
+        <v>40</v>
       </c>
       <c r="E39" s="46" t="s">
         <v>56</v>
       </c>
       <c r="F39" s="31">
-        <v>0.34</v>
+        <v>0.16500000000000001</v>
       </c>
       <c r="G39" s="16"/>
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B40" s="35" t="s">
-        <v>75</v>
-      </c>
-      <c r="C40" s="18"/>
-      <c r="D40" s="18"/>
-      <c r="E40" s="42">
-        <f>SUMIF(E41:E42,"Done",F41:F42)</f>
-        <v>0.5</v>
-      </c>
-      <c r="F40" s="22"/>
-      <c r="G40" s="18"/>
+      <c r="B40" s="16"/>
+      <c r="C40" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="D40" s="34" t="s">
+        <v>40</v>
+      </c>
+      <c r="E40" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="F40" s="31">
+        <v>0.16500000000000001</v>
+      </c>
+      <c r="G40" s="16"/>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B41" s="16"/>
-      <c r="C41" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="D41" s="16"/>
-      <c r="E41" s="46" t="s">
-        <v>56</v>
-      </c>
-      <c r="F41" s="31">
-        <v>0.5</v>
-      </c>
+      <c r="C41" s="34"/>
+      <c r="D41" s="34"/>
+      <c r="E41" s="46"/>
+      <c r="F41" s="31"/>
       <c r="G41" s="16"/>
     </row>
     <row r="42" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B42" s="16"/>
-      <c r="C42" s="34" t="s">
-        <v>95</v>
-      </c>
-      <c r="D42" s="34" t="s">
-        <v>145</v>
-      </c>
-      <c r="E42" s="40" t="s">
-        <v>144</v>
-      </c>
-      <c r="F42" s="31">
-        <v>0.5</v>
-      </c>
-      <c r="G42" s="16" t="s">
-        <v>146</v>
-      </c>
+      <c r="B42" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="C42" s="18"/>
+      <c r="D42" s="18"/>
+      <c r="E42" s="42">
+        <f>SUMIF(E43:E46,"Done",F43:F46)</f>
+        <v>0</v>
+      </c>
+      <c r="F42" s="22"/>
+      <c r="G42" s="18"/>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B43" s="35" t="s">
-        <v>76</v>
-      </c>
-      <c r="C43" s="18"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="42">
-        <f>SUMIF(E44:E45,"Done",F44:F45)</f>
-        <v>1</v>
-      </c>
-      <c r="F43" s="18"/>
-      <c r="G43" s="18"/>
+      <c r="B43" s="16"/>
+      <c r="C43" s="34" t="s">
+        <v>89</v>
+      </c>
+      <c r="D43" s="34" t="s">
+        <v>137</v>
+      </c>
+      <c r="E43" s="46" t="s">
+        <v>58</v>
+      </c>
+      <c r="F43" s="31">
+        <v>0.25</v>
+      </c>
+      <c r="G43" s="16" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="44" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B44" s="16"/>
       <c r="C44" s="34" t="s">
-        <v>96</v>
-      </c>
-      <c r="D44" s="16"/>
-      <c r="E44" s="46" t="s">
-        <v>56</v>
+        <v>148</v>
+      </c>
+      <c r="D44" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="E44" s="40" t="s">
+        <v>146</v>
       </c>
       <c r="F44" s="31">
-        <v>0.5</v>
-      </c>
-      <c r="G44" s="16"/>
+        <v>0.25</v>
+      </c>
+      <c r="G44" s="16" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B45" s="16"/>
       <c r="C45" s="34" t="s">
-        <v>97</v>
+        <v>149</v>
       </c>
       <c r="D45" s="34" t="s">
-        <v>99</v>
-      </c>
-      <c r="E45" s="46" t="s">
-        <v>56</v>
+        <v>1</v>
+      </c>
+      <c r="E45" s="40" t="s">
+        <v>136</v>
       </c>
       <c r="F45" s="31">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="G45" s="16"/>
     </row>
     <row r="46" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B46" s="35" t="s">
-        <v>127</v>
-      </c>
-      <c r="C46" s="18"/>
-      <c r="D46" s="18"/>
-      <c r="E46" s="41">
-        <f>SUMIF(E47:E47,"Done",F47:F47)</f>
+      <c r="B46" s="16"/>
+      <c r="C46" s="34" t="s">
+        <v>145</v>
+      </c>
+      <c r="D46" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="F46" s="53"/>
-      <c r="G46" s="18"/>
+      <c r="E46" s="40"/>
+      <c r="F46" s="31">
+        <v>0.25</v>
+      </c>
+      <c r="G46" s="16"/>
     </row>
     <row r="47" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B47" s="16"/>
-      <c r="C47" s="34" t="s">
-        <v>142</v>
-      </c>
+      <c r="C47" s="16"/>
       <c r="D47" s="16"/>
-      <c r="E47" s="46" t="s">
+      <c r="E47" s="16"/>
+      <c r="F47" s="16"/>
+      <c r="G47" s="16"/>
+    </row>
+    <row r="48" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B48" s="35" t="s">
+        <v>75</v>
+      </c>
+      <c r="C48" s="18"/>
+      <c r="D48" s="18"/>
+      <c r="E48" s="42">
+        <f>SUMIF(E49:E50,"Done",F49:F50)</f>
+        <v>1</v>
+      </c>
+      <c r="F48" s="18"/>
+      <c r="G48" s="18"/>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B49" s="16"/>
+      <c r="C49" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="D49" s="16"/>
+      <c r="E49" s="46" t="s">
         <v>56</v>
       </c>
-      <c r="F47" s="50">
+      <c r="F49" s="31">
+        <v>0.5</v>
+      </c>
+      <c r="G49" s="16"/>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B50" s="16"/>
+      <c r="C50" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="D50" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="E50" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="F50" s="31">
+        <v>0.5</v>
+      </c>
+      <c r="G50" s="16"/>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B51" s="16"/>
+      <c r="C51" s="34"/>
+      <c r="D51" s="34"/>
+      <c r="E51" s="46"/>
+      <c r="F51" s="31"/>
+      <c r="G51" s="16"/>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B52" s="35" t="s">
+        <v>120</v>
+      </c>
+      <c r="C52" s="18"/>
+      <c r="D52" s="18"/>
+      <c r="E52" s="41">
+        <f>SUMIF(E53:E53,"Done",F53:F53)</f>
         <v>1</v>
       </c>
-      <c r="G47" s="16"/>
-    </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B48" s="16"/>
-      <c r="C48" s="16"/>
-      <c r="D48" s="16"/>
-      <c r="E48" s="40"/>
-      <c r="F48" s="31"/>
-      <c r="G48" s="16"/>
-    </row>
-    <row r="49" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B49" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="C49" s="19"/>
-      <c r="D49" s="21"/>
-      <c r="E49" s="43">
-        <f>SUMIF(E50:E57,"Done",F50:F57)</f>
+      <c r="F52" s="53"/>
+      <c r="G52" s="18"/>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B53" s="16"/>
+      <c r="C53" s="34" t="s">
+        <v>134</v>
+      </c>
+      <c r="D53" s="16"/>
+      <c r="E53" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="F53" s="50">
+        <v>1</v>
+      </c>
+      <c r="G53" s="16"/>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B54" s="16"/>
+      <c r="C54" s="16"/>
+      <c r="D54" s="16"/>
+      <c r="E54" s="40"/>
+      <c r="F54" s="31"/>
+      <c r="G54" s="16"/>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B55" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="C55" s="19"/>
+      <c r="D55" s="21"/>
+      <c r="E55" s="43">
+        <f>SUMIF(E56:E63,"Done",F56:F63)</f>
         <v>0.86</v>
       </c>
-      <c r="F49" s="24"/>
-      <c r="G49" s="21"/>
-    </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B50" s="17"/>
-      <c r="C50" s="23" t="s">
-        <v>102</v>
-      </c>
-      <c r="D50" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="E50" s="49" t="s">
-        <v>56</v>
-      </c>
-      <c r="F50" s="32">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="G50" s="17" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B51" s="17"/>
-      <c r="C51" s="23" t="s">
-        <v>103</v>
-      </c>
-      <c r="D51" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="E51" s="44" t="s">
-        <v>56</v>
-      </c>
-      <c r="F51" s="32">
-        <v>0.12</v>
-      </c>
-      <c r="G51" s="17"/>
-    </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B52" s="17"/>
-      <c r="C52" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="D52" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="E52" s="44" t="s">
-        <v>56</v>
-      </c>
-      <c r="F52" s="32">
-        <v>0.12</v>
-      </c>
-      <c r="G52" s="23" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="53" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B53" s="17"/>
-      <c r="C53" s="23" t="s">
-        <v>105</v>
-      </c>
-      <c r="D53" s="23" t="s">
-        <v>2</v>
-      </c>
-      <c r="E53" s="44" t="s">
-        <v>56</v>
-      </c>
-      <c r="F53" s="32">
-        <v>0.12</v>
-      </c>
-      <c r="G53" s="17"/>
-    </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B54" s="17"/>
-      <c r="C54" s="23" t="s">
-        <v>106</v>
-      </c>
-      <c r="D54" s="23" t="s">
-        <v>2</v>
-      </c>
-      <c r="E54" s="44" t="s">
-        <v>56</v>
-      </c>
-      <c r="F54" s="32">
-        <v>0.12</v>
-      </c>
-      <c r="G54" s="17"/>
-    </row>
-    <row r="55" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B55" s="17"/>
-      <c r="C55" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="D55" s="23" t="s">
-        <v>2</v>
-      </c>
-      <c r="E55" s="44" t="s">
-        <v>56</v>
-      </c>
-      <c r="F55" s="32">
-        <v>0.12</v>
-      </c>
-      <c r="G55" s="23" t="s">
-        <v>116</v>
-      </c>
+      <c r="F55" s="24"/>
+      <c r="G55" s="21"/>
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B56" s="17"/>
       <c r="C56" s="23" t="s">
-        <v>123</v>
+        <v>96</v>
       </c>
       <c r="D56" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="E56" s="44" t="s">
+        <v>112</v>
+      </c>
+      <c r="E56" s="49" t="s">
         <v>56</v>
       </c>
       <c r="F56" s="32">
-        <v>0.12</v>
-      </c>
-      <c r="G56" s="23" t="s">
-        <v>125</v>
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="G56" s="17" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B57" s="17"/>
       <c r="C57" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="D57" s="23"/>
+        <v>97</v>
+      </c>
+      <c r="D57" s="23" t="s">
+        <v>112</v>
+      </c>
       <c r="E57" s="44" t="s">
-        <v>141</v>
+        <v>56</v>
       </c>
       <c r="F57" s="32">
         <v>0.12</v>
       </c>
-      <c r="G57" s="23"/>
+      <c r="G57" s="17"/>
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B58" s="17"/>
-      <c r="C58" s="23"/>
-      <c r="D58" s="23"/>
-      <c r="E58" s="44"/>
-      <c r="F58" s="32"/>
-      <c r="G58" s="23"/>
+      <c r="C58" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="D58" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="E58" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="F58" s="32">
+        <v>0.12</v>
+      </c>
+      <c r="G58" s="23" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B59" s="21" t="s">
-        <v>107</v>
-      </c>
-      <c r="C59" s="19"/>
-      <c r="D59" s="19"/>
-      <c r="E59" s="43">
-        <f>SUMIF(E60:E63,"Done",F60:F63)</f>
-        <v>1</v>
-      </c>
-      <c r="F59" s="24"/>
-      <c r="G59" s="19"/>
+      <c r="B59" s="17"/>
+      <c r="C59" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="D59" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="E59" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="F59" s="32">
+        <v>0.12</v>
+      </c>
+      <c r="G59" s="17"/>
     </row>
     <row r="60" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B60" s="17"/>
       <c r="C60" s="23" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="D60" s="23" t="s">
-        <v>1</v>
-      </c>
-      <c r="E60" s="49" t="s">
+        <v>2</v>
+      </c>
+      <c r="E60" s="44" t="s">
         <v>56</v>
       </c>
-      <c r="F60" s="33">
-        <v>0.25</v>
+      <c r="F60" s="32">
+        <v>0.12</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B61" s="17"/>
       <c r="C61" s="23" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D61" s="23" t="s">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E61" s="44" t="s">
         <v>56</v>
       </c>
-      <c r="F61" s="33">
-        <v>0.25</v>
-      </c>
-      <c r="G61" s="17"/>
+      <c r="F61" s="32">
+        <v>0.12</v>
+      </c>
+      <c r="G61" s="23" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="62" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B62" s="17"/>
       <c r="C62" s="23" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="D62" s="23" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="E62" s="44" t="s">
         <v>56</v>
       </c>
-      <c r="F62" s="33">
-        <v>0.25</v>
-      </c>
-      <c r="G62" s="17"/>
+      <c r="F62" s="32">
+        <v>0.12</v>
+      </c>
+      <c r="G62" s="23" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="63" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B63" s="17"/>
       <c r="C63" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="D63" s="23" t="s">
-        <v>1</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="D63" s="23"/>
       <c r="E63" s="44" t="s">
-        <v>56</v>
-      </c>
-      <c r="F63" s="33">
-        <v>0.25</v>
-      </c>
-      <c r="G63" s="17"/>
+        <v>133</v>
+      </c>
+      <c r="F63" s="32">
+        <v>0.12</v>
+      </c>
+      <c r="G63" s="23"/>
     </row>
     <row r="64" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B64" s="17"/>
-      <c r="C64" s="17"/>
-      <c r="D64" s="17"/>
-      <c r="E64" s="51"/>
-      <c r="F64" s="33"/>
-      <c r="G64" s="17"/>
+      <c r="C64" s="23"/>
+      <c r="D64" s="23"/>
+      <c r="E64" s="44"/>
+      <c r="F64" s="32"/>
+      <c r="G64" s="23"/>
     </row>
     <row r="65" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B65" s="21" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C65" s="19"/>
       <c r="D65" s="19"/>
       <c r="E65" s="43">
-        <f>SUMIF(E66:E67,"Done",F66:F67)</f>
+        <f>SUMIF(E66:E69,"Done",F66:F69)</f>
         <v>1</v>
       </c>
       <c r="F65" s="24"/>
@@ -2796,7 +2918,7 @@
     <row r="66" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B66" s="17"/>
       <c r="C66" s="23" t="s">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="D66" s="23" t="s">
         <v>1</v>
@@ -2805,48 +2927,133 @@
         <v>56</v>
       </c>
       <c r="F66" s="33">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="G66" s="17"/>
     </row>
     <row r="67" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B67" s="17"/>
       <c r="C67" s="23" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="D67" s="23" t="s">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="E67" s="44" t="s">
         <v>56</v>
       </c>
       <c r="F67" s="33">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="G67" s="17"/>
     </row>
     <row r="68" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B68" s="17"/>
-      <c r="C68" s="17"/>
-      <c r="D68" s="17"/>
-      <c r="E68" s="48"/>
-      <c r="F68" s="33"/>
+      <c r="C68" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="D68" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="E68" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="F68" s="33">
+        <v>0.25</v>
+      </c>
       <c r="G68" s="17"/>
     </row>
     <row r="69" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="F69"/>
+      <c r="B69" s="17"/>
+      <c r="C69" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="D69" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="E69" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="F69" s="33">
+        <v>0.25</v>
+      </c>
+      <c r="G69" s="17"/>
     </row>
     <row r="70" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="F70"/>
+      <c r="B70" s="17"/>
+      <c r="C70" s="17"/>
+      <c r="D70" s="17"/>
+      <c r="E70" s="51"/>
+      <c r="F70" s="33"/>
+      <c r="G70" s="17"/>
     </row>
     <row r="71" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="F71"/>
+      <c r="B71" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="C71" s="19"/>
+      <c r="D71" s="19"/>
+      <c r="E71" s="43">
+        <f>SUMIF(E72:E73,"Done",F72:F73)</f>
+        <v>1</v>
+      </c>
+      <c r="F71" s="24"/>
+      <c r="G71" s="19"/>
     </row>
     <row r="72" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="F72"/>
+      <c r="B72" s="17"/>
+      <c r="C72" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="D72" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="E72" s="49" t="s">
+        <v>56</v>
+      </c>
+      <c r="F72" s="33">
+        <v>0.5</v>
+      </c>
+      <c r="G72" s="17"/>
     </row>
     <row r="73" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="F73"/>
+      <c r="B73" s="17"/>
+      <c r="C73" s="23" t="s">
+        <v>114</v>
+      </c>
+      <c r="D73" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="E73" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="F73" s="33">
+        <v>0.5</v>
+      </c>
+      <c r="G73" s="17"/>
+    </row>
+    <row r="74" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B74" s="17"/>
+      <c r="C74" s="17"/>
+      <c r="D74" s="17"/>
+      <c r="E74" s="48"/>
+      <c r="F74" s="33"/>
+      <c r="G74" s="17"/>
+    </row>
+    <row r="75" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="F75"/>
+    </row>
+    <row r="76" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="F76"/>
+    </row>
+    <row r="77" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="F77"/>
+    </row>
+    <row r="78" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="F78"/>
+    </row>
+    <row r="79" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="F79"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2860,4 +3067,258 @@
     <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50B9F3C1-97AB-487F-B649-A50FE5815C35}">
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="27.33203125" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" customWidth="1"/>
+    <col min="4" max="4" width="23.21875" customWidth="1"/>
+    <col min="6" max="6" width="23" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1" t="s">
+        <v>181</v>
+      </c>
+      <c r="C1" t="s">
+        <v>182</v>
+      </c>
+      <c r="D1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="60" t="s">
+        <v>151</v>
+      </c>
+      <c r="C2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="60" t="s">
+        <v>152</v>
+      </c>
+      <c r="C3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="60" t="s">
+        <v>156</v>
+      </c>
+      <c r="C4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C5" t="s">
+        <v>173</v>
+      </c>
+      <c r="D5" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" s="60" t="s">
+        <v>155</v>
+      </c>
+      <c r="C6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D6" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B7" s="60"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>2</v>
+      </c>
+      <c r="B8" s="60" t="s">
+        <v>160</v>
+      </c>
+      <c r="C8" t="s">
+        <v>175</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9" s="60" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10" s="60" t="s">
+        <v>162</v>
+      </c>
+      <c r="C10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>3</v>
+      </c>
+      <c r="B11" s="60" t="s">
+        <v>163</v>
+      </c>
+      <c r="C11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B12" s="60"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>2</v>
+      </c>
+      <c r="B13" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="C13" s="60" t="s">
+        <v>176</v>
+      </c>
+      <c r="D13" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>3</v>
+      </c>
+      <c r="B14" s="60" t="s">
+        <v>164</v>
+      </c>
+      <c r="C14" t="s">
+        <v>153</v>
+      </c>
+      <c r="D14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>3</v>
+      </c>
+      <c r="B15" s="60" t="s">
+        <v>166</v>
+      </c>
+      <c r="C15" t="s">
+        <v>153</v>
+      </c>
+      <c r="D15" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>3</v>
+      </c>
+      <c r="B16" s="60" t="s">
+        <v>167</v>
+      </c>
+      <c r="C16" t="s">
+        <v>153</v>
+      </c>
+      <c r="D16" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B17" s="60"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>2</v>
+      </c>
+      <c r="B18" s="60" t="s">
+        <v>168</v>
+      </c>
+      <c r="C18" t="s">
+        <v>177</v>
+      </c>
+      <c r="D18" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>3</v>
+      </c>
+      <c r="B19" s="60" t="s">
+        <v>169</v>
+      </c>
+      <c r="C19" s="60" t="s">
+        <v>178</v>
+      </c>
+      <c r="D19" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>3</v>
+      </c>
+      <c r="B20" s="60" t="s">
+        <v>170</v>
+      </c>
+      <c r="C20" s="60" t="s">
+        <v>179</v>
+      </c>
+      <c r="D20" t="s">
+        <v>165</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update PCB V3 + Gestion de Projet
</commit_message>
<xml_diff>
--- a/#000 Coupe NI/Gestion_de_projet RACI Weekly.xlsx
+++ b/#000 Coupe NI/Gestion_de_projet RACI Weekly.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\ROBOT NI CONTEST\robotni\#000 Coupe NI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9234464C-36CA-49A6-9E0D-08446F404540}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC69375-6218-4070-9095-2EEBA04F2AD2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="705" activeTab="3" xr2:uid="{DA5DF307-7034-4F4E-90E0-F0D7D509C38B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="705" activeTab="2" xr2:uid="{DA5DF307-7034-4F4E-90E0-F0D7D509C38B}"/>
   </bookViews>
   <sheets>
     <sheet name="RACI" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,6 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="183">
   <si>
     <t xml:space="preserve">Semaine </t>
   </si>
@@ -472,9 +471,6 @@
   </si>
   <si>
     <t>#164 - Faire imprimer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analise </t>
   </si>
   <si>
     <t>Attente de la fin de l'analise</t>
@@ -906,13 +902,13 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="20 % - Accent1" xfId="3" builtinId="30"/>
@@ -1781,7 +1777,7 @@
         <v>138</v>
       </c>
       <c r="AE2" s="56" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:32" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1872,7 +1868,7 @@
         <v>131</v>
       </c>
       <c r="AE3" s="56" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4" spans="1:32" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1957,10 +1953,10 @@
         <v>131</v>
       </c>
       <c r="AD4" s="56" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AE4" s="56" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:32" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2029,7 +2025,7 @@
         <v>131</v>
       </c>
       <c r="AE5" s="56" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.3">
@@ -2072,18 +2068,18 @@
     <col min="2" max="2" width="28.109375" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
     <col min="4" max="4" width="29.88671875" customWidth="1"/>
-    <col min="6" max="6" width="8.6640625" style="26" customWidth="1"/>
+    <col min="6" max="6" width="8.6640625" style="26" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="35" customWidth="1"/>
     <col min="8" max="8" width="11.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="60" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
     </row>
     <row r="3" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B3" s="27" t="s">
@@ -2103,7 +2099,7 @@
       </c>
       <c r="C4" s="45">
         <f ca="1">(SUM(E10,C5,E15))/3</f>
-        <v>0.56285714285714283</v>
+        <v>0.5747619047619047</v>
       </c>
       <c r="D4" s="36" t="s">
         <v>135</v>
@@ -2115,7 +2111,7 @@
       </c>
       <c r="C5" s="41">
         <f>(SUM(E22,E26,E30,E34,E42,E18,E48))/7</f>
-        <v>0.68857142857142861</v>
+        <v>0.72428571428571431</v>
       </c>
       <c r="D5" s="18"/>
     </row>
@@ -2132,12 +2128,12 @@
       </c>
     </row>
     <row r="8" spans="2:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="58" t="s">
+      <c r="B8" s="59" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="58"/>
-      <c r="D8" s="58"/>
-      <c r="E8" s="58"/>
+      <c r="C8" s="59"/>
+      <c r="D8" s="59"/>
+      <c r="E8" s="59"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
@@ -2582,7 +2578,7 @@
       <c r="D42" s="18"/>
       <c r="E42" s="42">
         <f>SUMIF(E43:E46,"Done",F43:F46)</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="F42" s="22"/>
       <c r="G42" s="18"/>
@@ -2602,19 +2598,19 @@
         <v>0.25</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="44" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B44" s="16"/>
       <c r="C44" s="34" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D44" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="E44" s="40" t="s">
-        <v>146</v>
+      <c r="E44" s="46" t="s">
+        <v>56</v>
       </c>
       <c r="F44" s="31">
         <v>0.25</v>
@@ -2626,7 +2622,7 @@
     <row r="45" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B45" s="16"/>
       <c r="C45" s="34" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D45" s="34" t="s">
         <v>1</v>
@@ -3082,27 +3078,27 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B1" t="s">
         <v>180</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>181</v>
       </c>
-      <c r="C1" t="s">
-        <v>182</v>
-      </c>
       <c r="D1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="60" t="s">
-        <v>151</v>
+      <c r="B2" s="58" t="s">
+        <v>150</v>
       </c>
       <c r="C2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D2" t="s">
         <v>1</v>
@@ -3112,11 +3108,11 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="60" t="s">
+      <c r="B3" s="58" t="s">
+        <v>151</v>
+      </c>
+      <c r="C3" t="s">
         <v>152</v>
-      </c>
-      <c r="C3" t="s">
-        <v>153</v>
       </c>
       <c r="D3" t="s">
         <v>1</v>
@@ -3126,11 +3122,11 @@
       <c r="A4">
         <v>2</v>
       </c>
-      <c r="B4" s="60" t="s">
-        <v>156</v>
+      <c r="B4" s="58" t="s">
+        <v>155</v>
       </c>
       <c r="C4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D4" t="s">
         <v>1</v>
@@ -3140,42 +3136,42 @@
       <c r="A5">
         <v>2</v>
       </c>
-      <c r="B5" s="60" t="s">
-        <v>157</v>
+      <c r="B5" s="58" t="s">
+        <v>156</v>
       </c>
       <c r="C5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2</v>
       </c>
-      <c r="B6" s="60" t="s">
-        <v>155</v>
+      <c r="B6" s="58" t="s">
+        <v>154</v>
       </c>
       <c r="C6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B7" s="60"/>
+      <c r="B7" s="58"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2</v>
       </c>
-      <c r="B8" s="60" t="s">
-        <v>160</v>
+      <c r="B8" s="58" t="s">
+        <v>159</v>
       </c>
       <c r="C8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D8" t="s">
         <v>1</v>
@@ -3185,106 +3181,106 @@
       <c r="A9">
         <v>3</v>
       </c>
-      <c r="B9" s="60" t="s">
-        <v>161</v>
+      <c r="B9" s="58" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>3</v>
       </c>
-      <c r="B10" s="60" t="s">
-        <v>162</v>
+      <c r="B10" s="58" t="s">
+        <v>161</v>
       </c>
       <c r="C10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>3</v>
       </c>
-      <c r="B11" s="60" t="s">
-        <v>163</v>
+      <c r="B11" s="58" t="s">
+        <v>162</v>
       </c>
       <c r="C11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D11" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B12" s="60"/>
+      <c r="B12" s="58"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2</v>
       </c>
-      <c r="B13" s="60" t="s">
+      <c r="B13" s="58" t="s">
+        <v>157</v>
+      </c>
+      <c r="C13" s="58" t="s">
+        <v>175</v>
+      </c>
+      <c r="D13" t="s">
         <v>158</v>
-      </c>
-      <c r="C13" s="60" t="s">
-        <v>176</v>
-      </c>
-      <c r="D13" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>3</v>
       </c>
-      <c r="B14" s="60" t="s">
+      <c r="B14" s="58" t="s">
+        <v>163</v>
+      </c>
+      <c r="C14" t="s">
+        <v>152</v>
+      </c>
+      <c r="D14" t="s">
         <v>164</v>
-      </c>
-      <c r="C14" t="s">
-        <v>153</v>
-      </c>
-      <c r="D14" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>3</v>
       </c>
-      <c r="B15" s="60" t="s">
-        <v>166</v>
+      <c r="B15" s="58" t="s">
+        <v>165</v>
       </c>
       <c r="C15" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D15" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>3</v>
       </c>
-      <c r="B16" s="60" t="s">
-        <v>167</v>
+      <c r="B16" s="58" t="s">
+        <v>166</v>
       </c>
       <c r="C16" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D16" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="60"/>
+      <c r="B17" s="58"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2</v>
       </c>
-      <c r="B18" s="60" t="s">
-        <v>168</v>
+      <c r="B18" s="58" t="s">
+        <v>167</v>
       </c>
       <c r="C18" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D18" t="s">
         <v>2</v>
@@ -3294,28 +3290,28 @@
       <c r="A19">
         <v>3</v>
       </c>
-      <c r="B19" s="60" t="s">
-        <v>169</v>
-      </c>
-      <c r="C19" s="60" t="s">
-        <v>178</v>
+      <c r="B19" s="58" t="s">
+        <v>168</v>
+      </c>
+      <c r="C19" s="58" t="s">
+        <v>177</v>
       </c>
       <c r="D19" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>3</v>
       </c>
-      <c r="B20" s="60" t="s">
-        <v>170</v>
-      </c>
-      <c r="C20" s="60" t="s">
-        <v>179</v>
+      <c r="B20" s="58" t="s">
+        <v>169</v>
+      </c>
+      <c r="C20" s="58" t="s">
+        <v>178</v>
       </c>
       <c r="D20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto stash before merge of "Dev" and "origin/Dev"
</commit_message>
<xml_diff>
--- a/#000 Coupe NI/Gestion_de_projet RACI Weekly.xlsx
+++ b/#000 Coupe NI/Gestion_de_projet RACI Weekly.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\ROBOT NI CONTEST\robotni\#000 Coupe NI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC7F3F9-9FD1-41E3-9B22-57404C62D351}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C161F95F-0E1B-4382-8DDE-E6CA87BC1589}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="705" activeTab="2" xr2:uid="{DA5DF307-7034-4F4E-90E0-F0D7D509C38B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="705" xr2:uid="{DA5DF307-7034-4F4E-90E0-F0D7D509C38B}"/>
   </bookViews>
   <sheets>
     <sheet name="RACI" sheetId="2" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="198">
   <si>
     <t xml:space="preserve">Semaine </t>
   </si>
@@ -209,6 +209,9 @@
     <t>Teste/Reparation du raspberry</t>
   </si>
   <si>
+    <t>Freez</t>
+  </si>
+  <si>
     <t>Avencement du Projet</t>
   </si>
   <si>
@@ -440,6 +443,9 @@
     <t>IMPORTANT: ABSENCE DE REGLES NI</t>
   </si>
   <si>
+    <t>Quentin BAUDIN -&gt; Jason PUEL</t>
+  </si>
+  <si>
     <t>PCB V3</t>
   </si>
   <si>
@@ -464,6 +470,9 @@
     <t>#164 - Faire imprimer</t>
   </si>
   <si>
+    <t>Attente de la fin de l'analise</t>
+  </si>
+  <si>
     <t>#162 - Correction et amelioration</t>
   </si>
   <si>
@@ -614,10 +623,10 @@
     <t>#111 - Code Concours RT</t>
   </si>
   <si>
-    <t>le concour étant supprimer et en l'absence de régles nous nous donnons les points</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Jason PUEL</t>
+    <t>On s'allou les point car le concour n'existe plus</t>
+  </si>
+  <si>
+    <t>Taches</t>
   </si>
 </sst>
 </file>
@@ -683,7 +692,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -796,6 +805,12 @@
         <bgColor theme="8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="7">
     <border>
@@ -889,7 +904,7 @@
     <xf numFmtId="0" fontId="3" fillId="16" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1011,6 +1026,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1031,7 +1047,7 @@
     <cellStyle name="Sortie" xfId="9" builtinId="21"/>
     <cellStyle name="Titre" xfId="2" builtinId="15"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="12">
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1040,6 +1056,313 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="8"/>
+        </top>
+        <bottom style="thin">
+          <color theme="8"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="8"/>
+        </top>
+        <bottom style="thin">
+          <color theme="8"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="8"/>
+        </top>
+        <bottom style="thin">
+          <color theme="8"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="8"/>
+        </top>
+        <bottom style="thin">
+          <color theme="8"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="8"/>
+        </top>
+        <bottom style="thin">
+          <color theme="8"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="8"/>
+        </top>
+        <bottom style="thin">
+          <color theme="8"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="8"/>
+          <bgColor theme="8"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1071,6 +1394,22 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{FEBAB067-BD3A-46B8-BDB1-AD530B196BE0}" name="Tableau4" displayName="Tableau4" ref="B24:H44" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="B24:H44" xr:uid="{E74284EA-3994-4DAA-94BD-7A4BC8254B33}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{4BCFA966-C0F8-40DA-924C-717323F9FE70}" name="Taches" dataDxfId="9" dataCellStyle="20 % - Accent6"/>
+    <tableColumn id="2" xr3:uid="{CD6CF48E-59F0-4CDC-8E5F-CFE4C7E4AB1B}" name="Jason PUEL" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{B8C9200D-E960-49D2-87BD-083084DD54F9}" name="Christian Margolis" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{BECE3050-27B2-451E-B4ED-C72750CE9083}" name="Justin Furio" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{E7BF11CD-913F-474A-906C-53DCABB7D870}" name="Florian Guigal" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{731A2E17-6FBD-425B-BBCF-289C9545473B}" name="M2" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{B97D253C-EA36-45B5-9DAC-C2021AFA4A57}" name="Tuteur" dataDxfId="3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{32F8ADCA-7BE8-4A17-965F-3A7BAA9A6A31}" name="Tableau2" displayName="Tableau2" ref="B9:G74" totalsRowShown="0">
   <autoFilter ref="B9:G74" xr:uid="{5E9D7C67-1BBD-465F-A208-D11E9B7D938B}"/>
   <tableColumns count="6">
@@ -1085,7 +1424,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B234A6B6-6CB4-4E0A-BCEA-2089E7E950E6}" name="Tableau3" displayName="Tableau3" ref="B3:D6" totalsRowShown="0" headerRowDxfId="1" headerRowCellStyle="Sortie">
   <autoFilter ref="B3:D6" xr:uid="{F68388F4-7AF2-46C9-9F3D-5B6FB6A3583F}"/>
   <tableColumns count="3">
@@ -1395,13 +1734,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F51B35F8-C2A1-4A6B-AA0B-6756C7080F68}">
   <sheetPr codeName="Feuil1"/>
-  <dimension ref="B4:H49"/>
+  <dimension ref="B4:K44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="34.21875" customWidth="1"/>
     <col min="3" max="3" width="15.6640625" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
     <col min="5" max="5" width="16.5546875" customWidth="1"/>
     <col min="6" max="6" width="15.77734375" customWidth="1"/>
     <col min="7" max="7" width="15.6640625" customWidth="1"/>
@@ -1631,7 +1970,7 @@
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C17" s="7" t="s">
         <v>43</v>
       </c>
@@ -1639,7 +1978,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C18" s="11" t="s">
         <v>41</v>
       </c>
@@ -1647,7 +1986,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C19" s="13" t="s">
         <v>44</v>
       </c>
@@ -1655,7 +1994,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C20" s="9" t="s">
         <v>42</v>
       </c>
@@ -1663,7 +2002,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:11" x14ac:dyDescent="0.3">
       <c r="C21" s="5" t="s">
         <v>46</v>
       </c>
@@ -1671,7 +2010,10 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>197</v>
+      </c>
       <c r="C24" s="62" t="s">
         <v>1</v>
       </c>
@@ -1688,12 +2030,18 @@
         <v>39</v>
       </c>
       <c r="H24" s="64" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
+        <v>193</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="K24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B25" s="59" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>44</v>
@@ -1707,13 +2055,20 @@
       <c r="F25" s="65" t="s">
         <v>43</v>
       </c>
+      <c r="G25" s="67"/>
       <c r="H25" s="11" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="J25" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="K25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B26" s="59" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C26" s="63" t="s">
         <v>42</v>
@@ -1730,10 +2085,16 @@
       <c r="H26" s="63" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="J26" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="K26" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B27" s="59" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C27" s="65" t="s">
         <v>43</v>
@@ -1747,13 +2108,20 @@
       <c r="F27" s="63" t="s">
         <v>42</v>
       </c>
+      <c r="G27" s="67"/>
       <c r="H27" s="11" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="J27" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="K27" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B28" s="66" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C28" s="65" t="s">
         <v>43</v>
@@ -1771,9 +2139,9 @@
         <v>41</v>
       </c>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B29" s="60" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C29" s="65" t="s">
         <v>43</v>
@@ -1787,13 +2155,14 @@
       <c r="F29" s="65" t="s">
         <v>43</v>
       </c>
+      <c r="G29" s="67"/>
       <c r="H29" s="11" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B30" s="60" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C30" s="63" t="s">
         <v>42</v>
@@ -1814,9 +2183,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B31" s="60" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C31" s="63" t="s">
         <v>42</v>
@@ -1837,9 +2206,9 @@
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B32" s="60" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C32" s="65" t="s">
         <v>43</v>
@@ -1862,7 +2231,7 @@
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B33" s="60" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C33" s="63" t="s">
         <v>42</v>
@@ -1885,7 +2254,7 @@
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B34" s="60" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C34" s="63" t="s">
         <v>42</v>
@@ -1908,7 +2277,7 @@
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B35" s="60" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C35" s="63" t="s">
         <v>42</v>
@@ -1922,10 +2291,12 @@
       <c r="F35" s="65" t="s">
         <v>43</v>
       </c>
+      <c r="G35" s="67"/>
+      <c r="H35" s="67"/>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B36" s="60" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C36" s="65" t="s">
         <v>43</v>
@@ -1945,7 +2316,7 @@
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B37" s="60" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C37" s="13" t="s">
         <v>44</v>
@@ -1968,7 +2339,7 @@
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B38" s="60" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C38" s="63" t="s">
         <v>42</v>
@@ -1991,7 +2362,7 @@
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B39" s="61" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C39" s="63" t="s">
         <v>42</v>
@@ -2014,7 +2385,7 @@
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B40" s="61" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C40" s="63" t="s">
         <v>42</v>
@@ -2037,7 +2408,7 @@
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B41" s="61" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C41" s="63" t="s">
         <v>42</v>
@@ -2060,7 +2431,7 @@
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B42" s="61" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C42" s="63" t="s">
         <v>42</v>
@@ -2077,7 +2448,7 @@
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B43" s="61" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="C43" s="65" t="s">
         <v>43</v>
@@ -2100,7 +2471,7 @@
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B44" s="61" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C44" s="65" t="s">
         <v>43</v>
@@ -2121,42 +2492,11 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C46" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D46" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C47" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="D47" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="48" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C48" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="D48" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="49" spans="3:4" x14ac:dyDescent="0.3">
-      <c r="C49" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D49" t="s">
-        <v>50</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
+  <tableParts count="2">
     <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2337,41 +2677,41 @@
         <v>29</v>
       </c>
       <c r="T2" s="52" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="Y2" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="Z2" s="56"/>
       <c r="AA2" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AB2" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AC2" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AD2" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="AE2" s="56" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="AF2" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" spans="1:32" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -2431,38 +2771,38 @@
         <v>29</v>
       </c>
       <c r="T3" s="52" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="W3" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="Y3" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="Z3" s="56"/>
       <c r="AA3" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AB3" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AC3" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AD3" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AE3" s="56" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:32" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2524,30 +2864,30 @@
         <v>29</v>
       </c>
       <c r="T4" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U4" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="W4" s="2"/>
       <c r="X4" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="Y4" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="Z4" s="56"/>
       <c r="AB4" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="AC4" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AD4" s="56" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="AE4" s="14" t="s">
         <v>11</v>
@@ -2591,7 +2931,7 @@
       </c>
       <c r="S5" s="55"/>
       <c r="T5" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U5" s="3" t="s">
         <v>31</v>
@@ -2600,32 +2940,32 @@
         <v>31</v>
       </c>
       <c r="W5" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="X5" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Y5" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Z5" s="56"/>
       <c r="AA5" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AB5" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AC5" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AD5" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AE5" s="56" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="AF5" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.3">
@@ -2674,40 +3014,40 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B2" s="68" t="s">
-        <v>58</v>
-      </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
+      <c r="B2" s="69" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
     </row>
     <row r="3" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B3" s="27" t="s">
         <v>52</v>
       </c>
       <c r="C3" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="27" t="s">
         <v>64</v>
-      </c>
-      <c r="D3" s="27" t="s">
-        <v>63</v>
       </c>
       <c r="E3" s="25"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B4" s="36" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C4" s="45">
         <f ca="1">(SUM(E10,C5,E15))/3</f>
-        <v>0.95238095238095244</v>
+        <v>0.61904761904761907</v>
       </c>
       <c r="D4" s="36" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B5" s="35" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C5" s="41">
         <f>(SUM(E22,E26,E30,E34,E42,E18,E48))/7</f>
@@ -2717,30 +3057,30 @@
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B6" s="21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C6" s="43">
         <f>(SUM(E71,E65,E55))/3</f>
         <v>0.95333333333333325</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="67" t="s">
+      <c r="B8" s="68" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="67"/>
-      <c r="D8" s="67"/>
-      <c r="E8" s="67"/>
+      <c r="C8" s="68"/>
+      <c r="D8" s="68"/>
+      <c r="E8" s="68"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>52</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
         <v>55</v>
@@ -2749,15 +3089,15 @@
         <v>53</v>
       </c>
       <c r="F9" s="26" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B10" s="36" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C10" s="20"/>
       <c r="D10" s="20"/>
@@ -2771,10 +3111,10 @@
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B11" s="15"/>
       <c r="C11" s="29" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E11" s="47" t="s">
         <v>56</v>
@@ -2787,10 +3127,10 @@
     <row r="12" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B12" s="15"/>
       <c r="C12" s="29" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E12" s="47" t="s">
         <v>56</v>
@@ -2803,7 +3143,7 @@
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B13" s="15"/>
       <c r="C13" s="29" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D13" s="29" t="s">
         <v>1</v>
@@ -2826,13 +3166,13 @@
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B15" s="36" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C15" s="20"/>
       <c r="D15" s="20"/>
       <c r="E15" s="39">
         <f>SUMIF(E16,"Done",F16)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" s="28"/>
       <c r="G15" s="20"/>
@@ -2841,16 +3181,16 @@
       <c r="B16" s="15"/>
       <c r="C16" s="15"/>
       <c r="D16" s="29" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E16" s="54" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F16" s="37">
         <v>1</v>
       </c>
       <c r="G16" s="29" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.3">
@@ -2863,7 +3203,7 @@
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B18" s="35" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C18" s="18"/>
       <c r="D18" s="18"/>
@@ -2877,10 +3217,10 @@
     <row r="19" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B19" s="16"/>
       <c r="C19" s="34" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E19" s="40" t="s">
         <v>56</v>
@@ -2893,10 +3233,10 @@
     <row r="20" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B20" s="16"/>
       <c r="C20" s="34" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D20" s="34" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E20" s="46" t="s">
         <v>56</v>
@@ -2916,7 +3256,7 @@
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B22" s="35" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C22" s="18"/>
       <c r="D22" s="18"/>
@@ -2930,7 +3270,7 @@
     <row r="23" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B23" s="16"/>
       <c r="C23" s="34" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D23" s="16"/>
       <c r="E23" s="40"/>
@@ -2942,7 +3282,7 @@
     <row r="24" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B24" s="16"/>
       <c r="C24" s="34" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D24" s="16"/>
       <c r="E24" s="40" t="s">
@@ -2963,7 +3303,7 @@
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B26" s="35" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C26" s="18"/>
       <c r="D26" s="18"/>
@@ -2977,7 +3317,7 @@
     <row r="27" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B27" s="16"/>
       <c r="C27" s="34" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D27" s="16"/>
       <c r="E27" s="40" t="s">
@@ -2991,7 +3331,7 @@
     <row r="28" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B28" s="16"/>
       <c r="C28" s="34" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D28" s="34" t="s">
         <v>1</v>
@@ -3014,7 +3354,7 @@
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B30" s="35" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C30" s="18"/>
       <c r="D30" s="18"/>
@@ -3028,7 +3368,7 @@
     <row r="31" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B31" s="16"/>
       <c r="C31" s="34" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D31" s="16"/>
       <c r="E31" s="40"/>
@@ -3040,7 +3380,7 @@
     <row r="32" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B32" s="16"/>
       <c r="C32" s="34" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D32" s="16"/>
       <c r="E32" s="40" t="s">
@@ -3061,7 +3401,7 @@
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B34" s="35" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C34" s="18"/>
       <c r="D34" s="18"/>
@@ -3075,11 +3415,9 @@
     <row r="35" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B35" s="16"/>
       <c r="C35" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="D35" s="34" t="s">
-        <v>91</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="D35" s="16"/>
       <c r="E35" s="46" t="s">
         <v>56</v>
       </c>
@@ -3091,10 +3429,10 @@
     <row r="36" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B36" s="16"/>
       <c r="C36" s="34" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D36" s="34" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E36" s="40" t="s">
         <v>56</v>
@@ -3107,10 +3445,10 @@
     <row r="37" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B37" s="16"/>
       <c r="C37" s="34" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D37" s="34" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E37" s="46" t="s">
         <v>56</v>
@@ -3123,7 +3461,7 @@
     <row r="38" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B38" s="16"/>
       <c r="C38" s="34" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D38" s="34" t="s">
         <v>40</v>
@@ -3139,7 +3477,7 @@
     <row r="39" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B39" s="16"/>
       <c r="C39" s="34" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D39" s="34" t="s">
         <v>40</v>
@@ -3155,7 +3493,7 @@
     <row r="40" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B40" s="16"/>
       <c r="C40" s="34" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D40" s="34" t="s">
         <v>40</v>
@@ -3178,7 +3516,7 @@
     </row>
     <row r="42" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B42" s="35" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C42" s="18"/>
       <c r="D42" s="18"/>
@@ -3192,10 +3530,10 @@
     <row r="43" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B43" s="16"/>
       <c r="C43" s="34" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D43" s="34" t="s">
-        <v>194</v>
+        <v>136</v>
       </c>
       <c r="E43" s="46" t="s">
         <v>56</v>
@@ -3203,12 +3541,14 @@
       <c r="F43" s="31">
         <v>0.25</v>
       </c>
-      <c r="G43" s="16"/>
+      <c r="G43" s="16" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="44" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B44" s="16"/>
       <c r="C44" s="34" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D44" s="34" t="s">
         <v>1</v>
@@ -3220,13 +3560,13 @@
         <v>0.25</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B45" s="16"/>
       <c r="C45" s="34" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D45" s="34" t="s">
         <v>1</v>
@@ -3242,7 +3582,7 @@
     <row r="46" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B46" s="16"/>
       <c r="C46" s="34" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D46" s="34" t="s">
         <v>1</v>
@@ -3265,7 +3605,7 @@
     </row>
     <row r="48" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B48" s="35" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C48" s="18"/>
       <c r="D48" s="18"/>
@@ -3279,7 +3619,7 @@
     <row r="49" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B49" s="16"/>
       <c r="C49" s="34" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D49" s="16"/>
       <c r="E49" s="46" t="s">
@@ -3293,10 +3633,10 @@
     <row r="50" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B50" s="16"/>
       <c r="C50" s="34" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D50" s="34" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E50" s="46" t="s">
         <v>56</v>
@@ -3316,7 +3656,7 @@
     </row>
     <row r="52" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B52" s="35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C52" s="18"/>
       <c r="D52" s="18"/>
@@ -3330,7 +3670,7 @@
     <row r="53" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B53" s="16"/>
       <c r="C53" s="34" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D53" s="16"/>
       <c r="E53" s="46" t="s">
@@ -3351,7 +3691,7 @@
     </row>
     <row r="55" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B55" s="21" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C55" s="19"/>
       <c r="D55" s="21"/>
@@ -3365,10 +3705,10 @@
     <row r="56" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B56" s="17"/>
       <c r="C56" s="23" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D56" s="23" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E56" s="49" t="s">
         <v>56</v>
@@ -3377,16 +3717,16 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="G56" s="17" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B57" s="17"/>
       <c r="C57" s="23" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D57" s="23" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E57" s="44" t="s">
         <v>56</v>
@@ -3399,10 +3739,10 @@
     <row r="58" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B58" s="17"/>
       <c r="C58" s="23" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D58" s="23" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E58" s="44" t="s">
         <v>56</v>
@@ -3411,16 +3751,16 @@
         <v>0.12</v>
       </c>
       <c r="G58" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B59" s="17"/>
       <c r="C59" s="23" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D59" s="23" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E59" s="44" t="s">
         <v>56</v>
@@ -3433,7 +3773,7 @@
     <row r="60" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B60" s="17"/>
       <c r="C60" s="23" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D60" s="23" t="s">
         <v>2</v>
@@ -3449,7 +3789,7 @@
     <row r="61" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B61" s="17"/>
       <c r="C61" s="23" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D61" s="23" t="s">
         <v>2</v>
@@ -3461,16 +3801,16 @@
         <v>0.12</v>
       </c>
       <c r="G61" s="23" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="62" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B62" s="17"/>
       <c r="C62" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D62" s="23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E62" s="44" t="s">
         <v>56</v>
@@ -3479,19 +3819,17 @@
         <v>0.12</v>
       </c>
       <c r="G62" s="23" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="63" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B63" s="17"/>
       <c r="C63" s="23" t="s">
-        <v>125</v>
-      </c>
-      <c r="D63" s="23" t="s">
-        <v>116</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="D63" s="23"/>
       <c r="E63" s="44" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F63" s="32">
         <v>0.12</v>
@@ -3508,7 +3846,7 @@
     </row>
     <row r="65" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B65" s="21" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C65" s="19"/>
       <c r="D65" s="19"/>
@@ -3522,7 +3860,7 @@
     <row r="66" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B66" s="17"/>
       <c r="C66" s="23" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D66" s="23" t="s">
         <v>1</v>
@@ -3538,7 +3876,7 @@
     <row r="67" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B67" s="17"/>
       <c r="C67" s="23" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D67" s="23" t="s">
         <v>40</v>
@@ -3554,10 +3892,10 @@
     <row r="68" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B68" s="17"/>
       <c r="C68" s="23" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D68" s="23" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E68" s="44" t="s">
         <v>56</v>
@@ -3570,7 +3908,7 @@
     <row r="69" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B69" s="17"/>
       <c r="C69" s="23" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D69" s="23" t="s">
         <v>1</v>
@@ -3593,7 +3931,7 @@
     </row>
     <row r="71" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B71" s="21" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C71" s="19"/>
       <c r="D71" s="19"/>
@@ -3607,7 +3945,7 @@
     <row r="72" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B72" s="17"/>
       <c r="C72" s="23" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D72" s="23" t="s">
         <v>1</v>
@@ -3623,7 +3961,7 @@
     <row r="73" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B73" s="17"/>
       <c r="C73" s="23" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D73" s="23" t="s">
         <v>1</v>
@@ -3686,16 +4024,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B1" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -3703,10 +4041,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="58" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D2" t="s">
         <v>1</v>
@@ -3717,10 +4055,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="58" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D3" t="s">
         <v>1</v>
@@ -3731,10 +4069,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="58" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C4" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D4" t="s">
         <v>1</v>
@@ -3745,13 +4083,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="58" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -3759,13 +4097,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="58" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D6" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -3776,10 +4114,10 @@
         <v>2</v>
       </c>
       <c r="B8" s="58" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C8" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D8" t="s">
         <v>1</v>
@@ -3790,7 +4128,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="58" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -3798,10 +4136,10 @@
         <v>3</v>
       </c>
       <c r="B10" s="58" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C10" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -3809,10 +4147,10 @@
         <v>3</v>
       </c>
       <c r="B11" s="58" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C11" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D11" t="s">
         <v>1</v>
@@ -3826,13 +4164,13 @@
         <v>2</v>
       </c>
       <c r="B13" s="58" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C13" s="58" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D13" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -3840,13 +4178,13 @@
         <v>3</v>
       </c>
       <c r="B14" s="58" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C14" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D14" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -3854,13 +4192,13 @@
         <v>3</v>
       </c>
       <c r="B15" s="58" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C15" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D15" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -3868,13 +4206,13 @@
         <v>3</v>
       </c>
       <c r="B16" s="58" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C16" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D16" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -3885,10 +4223,10 @@
         <v>2</v>
       </c>
       <c r="B18" s="58" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C18" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D18" t="s">
         <v>2</v>
@@ -3899,13 +4237,13 @@
         <v>3</v>
       </c>
       <c r="B19" s="58" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C19" s="58" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D19" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -3913,13 +4251,13 @@
         <v>3</v>
       </c>
       <c r="B20" s="58" t="s">
+        <v>164</v>
+      </c>
+      <c r="C20" s="58" t="s">
+        <v>170</v>
+      </c>
+      <c r="D20" t="s">
         <v>161</v>
-      </c>
-      <c r="C20" s="58" t="s">
-        <v>167</v>
-      </c>
-      <c r="D20" t="s">
-        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>